<commit_message>
Initial image and chart - not working
</commit_message>
<xml_diff>
--- a/config/g-slide mapping.xlsx
+++ b/config/g-slide mapping.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Valuation\Commercial\Valuer Resources\Forbury\G-Slide\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{504D367F-2EBC-400D-8E5B-63CEBE4726C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38599BD6-AC72-4A43-B5C4-A8571316DAC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AA2C21C5-C99D-45A6-8DBB-603319E3FB5B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{AA2C21C5-C99D-45A6-8DBB-603319E3FB5B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Tables" sheetId="2" r:id="rId2"/>
+    <sheet name="Graphs" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="118">
   <si>
     <t>Sheet Name</t>
   </si>
@@ -294,6 +296,102 @@
   </si>
   <si>
     <t>MktVSContractRentPercentDif1</t>
+  </si>
+  <si>
+    <t>PRP DCF</t>
+  </si>
+  <si>
+    <t>Z05_RunningYield_PRP</t>
+  </si>
+  <si>
+    <t>sheet_name</t>
+  </si>
+  <si>
+    <t>chart_name</t>
+  </si>
+  <si>
+    <t>bookmark_name</t>
+  </si>
+  <si>
+    <t>Z05_TenancyProfileByIncome_PRP</t>
+  </si>
+  <si>
+    <t>Z05_LeaseExpiryAreaTerminal_PRP</t>
+  </si>
+  <si>
+    <t>Z05_ProjectedNetCashflow_PRP</t>
+  </si>
+  <si>
+    <t>Chart_RunningYield_PRP1</t>
+  </si>
+  <si>
+    <t>Chart_ProjectedNetCashflow_PRP1</t>
+  </si>
+  <si>
+    <t>Chart_TenancyProfileByIncome_PRP1</t>
+  </si>
+  <si>
+    <t>Chart_LeaseExpiryAreaTerminal_PRP1</t>
+  </si>
+  <si>
+    <t>Chart_TenancyProfileByIncome_PRP2</t>
+  </si>
+  <si>
+    <t>Chart_LeaseExpiryAreaTerminal_PRP2</t>
+  </si>
+  <si>
+    <t>Chart_RunningYield_PRP2</t>
+  </si>
+  <si>
+    <t>Chart_ProjectedNetCashflow_PRP2</t>
+  </si>
+  <si>
+    <t>PRP MktCap</t>
+  </si>
+  <si>
+    <t>B7:I72</t>
+  </si>
+  <si>
+    <t>cell_range</t>
+  </si>
+  <si>
+    <t>PRP TenSched</t>
+  </si>
+  <si>
+    <t>B11:V21</t>
+  </si>
+  <si>
+    <t>Table_TenSched</t>
+  </si>
+  <si>
+    <t>Table_MarketCap</t>
+  </si>
+  <si>
+    <t>New Sales Table</t>
+  </si>
+  <si>
+    <t>B1:N22</t>
+  </si>
+  <si>
+    <t>Table_SalesTable</t>
+  </si>
+  <si>
+    <t>B7:M75</t>
+  </si>
+  <si>
+    <t>Table_DCF1</t>
+  </si>
+  <si>
+    <t>Table_DCF2</t>
+  </si>
+  <si>
+    <t>B77:M132</t>
+  </si>
+  <si>
+    <t>B2:F22</t>
+  </si>
+  <si>
+    <t>Table_ValSum</t>
   </si>
 </sst>
 </file>
@@ -1369,27 +1467,213 @@
 </worksheet>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99b60f7e-3057-4f81-988a-62a9628edd05">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="e25ec18d-f618-48a6-82de-2a1b818da741" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB222A80-7E8D-4A74-84FB-209271147ED0}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.85546875" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C5" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>116</v>
+      </c>
+      <c r="C7" t="s">
+        <v>117</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B4DEDD3-E66F-47BE-BC2C-F55A5342F695}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" t="s">
+        <v>92</v>
+      </c>
+      <c r="C7" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B8" t="s">
+        <v>91</v>
+      </c>
+      <c r="C8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>86</v>
+      </c>
+      <c r="B9" t="s">
+        <v>92</v>
+      </c>
+      <c r="C9" t="s">
+        <v>99</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002CE86911AAD3E04DBFE431D89A8CA577" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9aa131caeef7cdb6c57c83274dc12eab">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="99b60f7e-3057-4f81-988a-62a9628edd05" xmlns:ns3="e25ec18d-f618-48a6-82de-2a1b818da741" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="572a6d1f7b9f236d973fbfadd6951c98" ns2:_="" ns3:_="">
     <xsd:import namespace="99b60f7e-3057-4f81-988a-62a9628edd05"/>
@@ -1596,26 +1880,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235DF9EF-4EA4-4B67-A9D1-345F7233E7B1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="99b60f7e-3057-4f81-988a-62a9628edd05"/>
-    <ds:schemaRef ds:uri="e25ec18d-f618-48a6-82de-2a1b818da741"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3138D381-CBAD-4FB8-B98A-9D1E01DB5310}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="99b60f7e-3057-4f81-988a-62a9628edd05">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="e25ec18d-f618-48a6-82de-2a1b818da741" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E247AB3-8E74-4F26-8623-21341DBDF478}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1632,4 +1917,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3138D381-CBAD-4FB8-B98A-9D1E01DB5310}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{235DF9EF-4EA4-4B67-A9D1-345F7233E7B1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="99b60f7e-3057-4f81-988a-62a9628edd05"/>
+    <ds:schemaRef ds:uri="e25ec18d-f618-48a6-82de-2a1b818da741"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>